<commit_message>
update admin console 6,7 & base web mvc
</commit_message>
<xml_diff>
--- a/src/main/java/com/example/admissions_management/shared/docs/excels/Nguong dau vao 2025.xlsx
+++ b/src/main/java/com/example/admissions_management/shared/docs/excels/Nguong dau vao 2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Daotao_05_2023\01_Tuyen sinh\TS Nam 2025\08. Nguong dau vao\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MHPL\Admissions-Management-main\src\main\java\com\example\admissions_management\shared\docs\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B643B448-B6F4-4179-A949-EAB7418C736C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5DBE0B4-4300-4175-8790-A7E338AA00A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{106C5DE0-1326-4526-93C8-4EFC1FD5E8CA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{106C5DE0-1326-4526-93C8-4EFC1FD5E8CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -587,14 +585,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AD8E549-11A5-4ED3-A5AA-F2B24EFB58D2}">
   <dimension ref="A1:D48"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.85546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="59.85546875" customWidth="1"/>
-    <col min="4" max="4" width="21.5703125" customWidth="1"/>
+    <col min="2" max="2" width="13.88671875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="59.88671875" customWidth="1"/>
+    <col min="4" max="4" width="21.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -608,7 +606,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -622,7 +620,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -636,7 +634,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -650,7 +648,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -664,7 +662,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -678,7 +676,7 @@
         <v>24.5</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -692,7 +690,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -706,7 +704,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -720,7 +718,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -734,7 +732,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -748,7 +746,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -762,7 +760,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -776,7 +774,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -790,7 +788,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -804,7 +802,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -818,7 +816,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -832,7 +830,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -846,7 +844,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -860,7 +858,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -874,7 +872,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -888,7 +886,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -902,7 +900,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -916,7 +914,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -930,7 +928,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -944,7 +942,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -958,7 +956,7 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -972,7 +970,7 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -986,7 +984,7 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1000,7 +998,7 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1014,7 +1012,7 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1028,7 +1026,7 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1042,7 +1040,7 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1056,7 +1054,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1070,7 +1068,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1084,7 +1082,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1098,7 +1096,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1112,7 +1110,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1126,7 +1124,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1140,7 +1138,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1154,7 +1152,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1168,7 +1166,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1182,7 +1180,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1196,7 +1194,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1210,7 +1208,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1224,7 +1222,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1238,7 +1236,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1252,7 +1250,7 @@
         <v>20.5</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>

</xml_diff>